<commit_message>
deploy: 更新 GitHub Pages (2026-05-17 16:14)
</commit_message>
<xml_diff>
--- a/股癌_股票追蹤.xlsx
+++ b/股癌_股票追蹤.xlsx
@@ -673,20 +673,20 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>EP661</t>
+          <t>EP662</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>孟公將部分中小部位轉入台積電，持續持有</t>
+          <t>金管會放寬主動型ETF持股上限，預計1個月後投信陸續增持，籌碼面中期利多；資金輪動可能造成中小股賣壓</t>
         </is>
       </c>
     </row>
@@ -1483,20 +1483,20 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>EP659</t>
+          <t>EP662</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>軟體被殺中相對撐得住的標的之一</t>
+          <t>資安股逆勢創新高，Mythos負面衝擊未兌現反而拉升需求，AI時代網路安全支出持續增加</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4951,6 +4951,70 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>EP662</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>台積電</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>台股</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>金管會放寬主動型ETF持股上限，預計1個月後投信陸續增持，籌碼面中期利多；資金輪動可能造成中小股賣壓</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>EP662</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>CrowdStrike</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>美股</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>資安股逆勢創新高，Mythos負面衝擊未兌現反而拉升需求，AI時代網路安全支出持續增加</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
deploy: 更新 GitHub Pages (2026-05-20 17:10)
</commit_message>
<xml_diff>
--- a/股癌_股票追蹤.xlsx
+++ b/股癌_股票追蹤.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -673,20 +673,20 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>EP662</t>
+          <t>EP663</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>金管會放寬主動型ETF持股上限，預計1個月後投信陸續增持，籌碼面中期利多；資金輪動可能造成中小股賣壓</t>
+          <t>技術論壇揭露三層蛋糕光通架構，確認光通長期方向；有紀律擴產控制保護供需週期</t>
         </is>
       </c>
     </row>
@@ -763,20 +763,20 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>EP660</t>
+          <t>EP663</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>連續漲停後進處置，資金面限制引爭議，主持人認為機制應針對大型股調整</t>
+          <t>Broadcom AI晶片V7/V8/V9 Zebrafish系列合作夥伴；某一代代號消失，但供應鏈整體持續，屬老AI族群短期修正中</t>
         </is>
       </c>
     </row>
@@ -2622,6 +2622,51 @@
       <c r="I48" t="inlineStr">
         <is>
           <t>MCU+CPU socket，兩年前Google/微軟綁定故事重新被炒，近期補漲</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Broadcom</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>美股</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>EP663</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>EP663</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>SoundFish後推出更大顆雙拼版（兩片晶片放在同一載板），老AI短期資金撤退，產品線持續推進；長期故事未結束，等資金輪動回來</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5015,6 +5060,102 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>EP663</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Broadcom</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>美股</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>SoundFish後推出更大顆雙拼版（兩片晶片放在同一載板），老AI短期資金撤退，產品線持續推進；長期故事未結束，等資金輪動回來</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>EP663</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2454</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>聯發科</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>台股</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Broadcom AI晶片V7/V8/V9 Zebrafish系列合作夥伴；某一代代號消失，但供應鏈整體持續，屬老AI族群短期修正中</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>EP663</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>台積電</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>台股</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>技術論壇揭露三層蛋糕光通架構，確認光通長期方向；有紀律擴產控制保護供需週期</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>